<commit_message>
fix: limit survival inference and align submission wording
</commit_message>
<xml_diff>
--- a/supplementary_tables/Supplementary_Tables_S1-S8.xlsx
+++ b/supplementary_tables/Supplementary_Tables_S1-S8.xlsx
@@ -53,7 +53,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -84,8 +84,14 @@
       <color rgb="00203744"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="006D777B"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -100,6 +106,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F4F7F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDF0F1"/>
       </patternFill>
     </fill>
   </fills>
@@ -120,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -135,6 +146,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -526,10 +540,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="39" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Effect per one-unit higher ZEB balance. BH correction across six endpoints separately within each model. Full model uses endpoint-specific complete cases (see S4).</t>
+          <t>Effect per one-unit higher ZEB balance. BH correction across six endpoints within each model. EFS/OS P and FDR are retained as audit outputs only: fully adjusted Cox fits had sparse-subtype convergence warnings and do not support survival inference (see S4).</t>
         </is>
       </c>
     </row>
@@ -844,124 +858,124 @@
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Event-free survival</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>1309/217</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>0.84 (0.78–0.91)</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>1.84e-05</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>2.21e-05</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>0.90 (0.81–1.00)</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>0.0504</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>0.101</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="J8" s="6" t="inlineStr">
         <is>
           <t>0.88 (0.79–0.97)</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="K8" s="6" t="inlineStr">
         <is>
           <t>0.0142</t>
         </is>
       </c>
-      <c r="L8" s="4" t="inlineStr">
+      <c r="L8" s="6" t="inlineStr">
         <is>
           <t>0.0284</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Overall survival</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>1309/140</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>0.84 (0.76–0.92)</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>2.95e-04</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>2.95e-04</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>0.90 (0.79–1.03)</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>0.114</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>0.137</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="J9" s="6" t="inlineStr">
         <is>
           <t>0.86 (0.76–0.98)</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr">
+      <c r="K9" s="6" t="inlineStr">
         <is>
           <t>0.0273</t>
         </is>
       </c>
-      <c r="L9" s="5" t="inlineStr">
+      <c r="L9" s="6" t="inlineStr">
         <is>
           <t>0.041</t>
         </is>
@@ -1002,7 +1016,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="39" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Leave-one-marker-out scores and an expanded normal-direction marker set were fitted within the same diagnostic cohort. Expanded genes have only two normal-source directional checks; all are expression proxies.</t>
@@ -3459,7 +3473,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="39" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>The same 1,309 patients enter full fits; 1 singleton author-IP 'Other' sample is held in training for all CV models, leaving 1,308 held-out predictions per repeat. No patient contributes to both train and test within a fold.</t>
@@ -3720,7 +3734,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="39" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Three fixed pairwise median comparisons use 3,000 within-group patient bootstraps. The ETP match is deterministic one-to-one nearest-coordinate matching without replacement; matched-pair mean CI uses 3,000 pair bootstraps. No causal interpretation.</t>
@@ -5251,10 +5265,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="39" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Model includes 17-subtype indicators, age, sex and log10 white-cell count. PH columns apply only to Cox models; inspect sparse-subtype warnings in source data.</t>
+          <t>Model includes 17-subtype indicators, age, sex and log10 white-cell count. EFS/OS Cox fits had sparse-subtype convergence warnings: their P/FDR values are audit outputs only, not evidence of survival association. PH tests do not resolve convergence instability.</t>
         </is>
       </c>
     </row>
@@ -5494,96 +5508,96 @@
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Event-free survival</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Cox PH</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>1306/217</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>0.88 (0.79–0.97)</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>0.0142</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>0.0284</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>0.0643</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>0.136</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Loglik converged before variable  3,4,9 ; coefficient may be infinite. </t>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AUDIT ONLY — Loglik converged before variable  3,4,9 ; coefficient may be infinite. </t>
         </is>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Overall survival</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Cox PH</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>1306/140</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>0.86 (0.76–0.98)</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>0.0273</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>0.041</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>0.668</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>0.696</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Loglik converged before variable  3,4,9,10,12 ; coefficient may be infinite. </t>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AUDIT ONLY — Loglik converged before variable  3,4,9,10,12 ; coefficient may be infinite. </t>
         </is>
       </c>
     </row>
@@ -5697,7 +5711,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="28" customHeight="1">
+    <row r="4" ht="42" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>ZEB1</t>
@@ -5759,7 +5773,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1">
+    <row r="5" ht="42" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>ZEB2</t>
@@ -5821,7 +5835,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="28" customHeight="1">
+    <row r="6" ht="42" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>LMO2</t>
@@ -5883,7 +5897,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1">
+    <row r="7" ht="42" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>ZEB balance</t>

</xml_diff>